<commit_message>
fixing the extraction agent
</commit_message>
<xml_diff>
--- a/architecture-ai/backend/rapport.xlsx
+++ b/architecture-ai/backend/rapport.xlsx
@@ -50,12 +50,11 @@
     </font>
     <font>
       <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="001F4E79"/>
-      <sz val="10"/>
+      <color rgb="00000000"/>
+      <sz val="9"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -75,11 +74,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -109,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -120,6 +114,12 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -129,7 +129,13 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -497,91 +503,1006 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="38" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="35" customWidth="1" min="10" max="10"/>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DOSSIER TECHNIQUE AMIANTE — 22 rue des Panoyaux, Bat. A; Esc. 1; Etage 2, 75020 PARIS - 20EME</t>
+          <t>RAPPORT D'EXTRACTION — 2-4 rue Corot 91380 CHILLY-MAZARIN</t>
         </is>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Réf. dossier : 33153_6  |  Date repérage : 16/09/2024  |  Opérateur : DULIN Nicolas, Opérateur de repérage, BUREAU VERITAS CERTIFICATION France 1 place Zaha Hadid 92400 COURBEVOIE, Obtention : 31/05/2023 Échéance : 18/04/2030 N° de certification : 8053942 et 15476985  |  Labo : </t>
+          <t>Réf. dossier : RAAT-595-BAT-1109L-BAT-A_v1  |  Opérateur : Julien DETOUL Certificat délivré par ICERT CPDI 5590 V002 délivré le 17/06/2020 et expirant le 16/06/2027</t>
         </is>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>Localisation</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Tour</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Localisation</t>
+          <t>Reference echantillon</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Description du matériau</t>
+          <t>Localisation 2</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Composant</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Réf. Échantillon</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>Réf. Labo</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>Résultat</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>État de conservation</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>Préconisation</t>
+          <t>Resultat</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Bâtiment A - Toiture- terrasse</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Revêtement étanchéité</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Toiture/P33</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Sol</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Amiante non détecté</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Bâtiment A - Toiture- terrasse</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Revêtement étanchéité + isolant type mousse</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Toiture/P34</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Sol</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Amiante non détecté</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Bâtiment A - Toiture- terrasse</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Revêtement bitumineux pare vapeur</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Toiture/P35</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Sol</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Amiante non détecté</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Bâtiment A - Toiture- terrasse</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Remontée d'étanchéité pax alu</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Toiture/P36</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Mur</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Amiante non détecté</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Bâtiment A - extérieur</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Colle de carrelage + peinture</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>A/P01</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Façade avant</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Amiante non détecté</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Bâtiment A - entrée 4</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Calorifuge</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>A/P02</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Plafond R-1</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Amiante non détecté</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Bâtiment A - extérieur</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Enduit + peinture + isolant sur ITE</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>A/P03</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Pignon gauche</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Amiante non détecté</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Bâtiment A - entrée 4</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Enduit</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>A/P04</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Mur gaine technique R+3</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Amiante non détecté</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Bâtiment A - entrée 4</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Fibralith</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>A/P05</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Plafond cave</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Amiante non détecté</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Bâtiment A - extérieur</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Joint de dilatation</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>A/P06</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Façade avant</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Amiante non détecté</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Bâtiment A - entrée 2</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Enduit + peinture</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>A/P07</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Mur RDC</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Amiante non détecté</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Bâtiment A - entrée 2</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Enduit + peinture</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>A/P08</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Plafond RDC</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Amiante non détecté</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Bâtiment A - entrée 2</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Enduit + peinture</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>A/P09</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Sous-face escalier RDC</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Amiante non détecté</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Bâtiment A - entrée 2</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Enduit + peinture</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>A/P10</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Mur R+2</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Amiante non détecté</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Bâtiment A - entrée 2</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Enduit + peinture</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>A/P11</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Plafond r R+2</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Amiante non détecté</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Bâtiment A - entrée 2</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Enduit + peinture</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>A/P12</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Sous-face escalier R+2</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Amiante non détecté</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Bâtiment A - entrée 2</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Peinture</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>A/P13</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Garde-corps RDC</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Amiante non détecté</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Bâtiment A - entrée 2</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Enduit</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>A/P14</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Mur cave</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Amiante non détecté</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Bâtiment A - entrée 2</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Fibralith</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>A/P15</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Plafond cave</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>Amiante non détecté</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Bâtiment A - entrée 2</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Calorifuge</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>A/P16</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Plafond R-1</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Amiante non détecté</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Bâtiment A - entrée 2</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Enduit</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>A/P17</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Mur gaine technique R-1</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Amiante non détecté</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Bâtiment A - entrée 2</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Enduit + peinture</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>A/P18</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Mur local OM</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Amiante non détecté</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Bâtiment A - entrée 2</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Fibralith</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>A/P19</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>Plafond local OM</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>Amiante non détecté</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Bâtiment A - entrée 2</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Peinture</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>A/P20</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Sol local OM</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Amiante non détecté</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Bâtiment A - entrée 2</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Tampon bitumineux</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>A/P21</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>Trappe local OM</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>Amiante non détecté</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Bâtiment A - entrée 2</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Isolant type laine de verre</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>A/P22</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>Trappe local OM</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Amiante non détecté</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Bâtiment A - entrée 2</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Joint sur conduit</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>A/P23</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>Conduit vide-ordure local OM</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>Amiante non détecté</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Bâtiment A - entrée 4</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Enduit + peinture</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>A/P24</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Mur R+1</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>Amiante non détecté</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Bâtiment A - entrée 4</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Enduit + peinture</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>A/P25</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>Plafond R+1</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>Amiante non détecté</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Bâtiment A - entrée 4</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Enduit + peinture</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>A/P26</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Sous-face escalier R+1</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>Amiante non détecté</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Bâtiment A - entrée 4</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Enduit + peinture</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>A/P27</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>Mur R+3</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>Amiante non détecté</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="30" customHeight="1">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Bâtiment A - entrée 4</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Enduit + peinture</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>A/P28</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>Plafond R+3</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Amiante non détecté</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="30" customHeight="1">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Bâtiment A - entrée 4</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>Enduit + peinture</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>A/P29</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>Sous-face escalier R+3</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>Amiante non détecté</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Bâtiment A - entrée 4</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Peinture</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>A/P30</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Garde-corps R+3</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Amiante non détecté</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Bâtiment A - entrée 4</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Enduit</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>A/P31</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>Mur cave</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>Amiante non détecté</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -593,7 +1514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -604,82 +1525,125 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SYNTHÈSE — 22 rue des Panoyaux, Bat. A; Esc. 1; Etage 2, 75020 PARIS - 20EME</t>
+          <t>SYNTHÈSE — 2-4 rue Corot 91380 CHILLY-MAZARIN</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>INDICATEUR</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>VALEUR</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>COMMENTAIRE</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>Total matériaux analysés</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Total matériaux</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Matériaux avec présence d'amiante</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>Listes A et B confondues</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>Matériaux contenant de l'amiante</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>Présence confirmée</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Matériaux sans amiante</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>Absence confirmée</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>MATÉRIAUX AMIANTÉS PAR PRÉCONISATION</t>
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>CONFIGURATION D'EXTRACTION</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Pages extraites</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>11 → 11</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>Colonnes extraites</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>Localisation, Description, Reference de l'Echantillon, Localisation 2, RESULTAT</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>Telles qu'elles apparaissent dans le document source</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Champs normalisés</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>localisation, description, reference_echantillon, localisation_2, resultat</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>Noms des colonnes dans ce fichier Excel</t>
         </is>
       </c>
     </row>

</xml_diff>